<commit_message>
Actualizacion de carta gantt
</commit_message>
<xml_diff>
--- a/Capstone/Fase 1/Grupales/Carta Gantt.xlsx
+++ b/Capstone/Fase 1/Grupales/Carta Gantt.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF7B829F-2271-4064-9E93-AFEFBB24DB9B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5602A59B-C963-41E5-8259-2A8CD39AEB17}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1125" yWindow="1125" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Carta Gatt" sheetId="11" r:id="rId1"/>
@@ -1303,6 +1303,39 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="41" borderId="24" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="19" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="8">
+      <alignment horizontal="right" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="8" applyBorder="1">
+      <alignment horizontal="right" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="8" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="8" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="168" fontId="7" fillId="0" borderId="3" xfId="9">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="2" xfId="12" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="169" fontId="0" fillId="5" borderId="22" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1314,39 +1347,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="42" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="19" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="8">
-      <alignment horizontal="right" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="8" applyBorder="1">
-      <alignment horizontal="right" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="8" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="8" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
-    <xf numFmtId="168" fontId="7" fillId="0" borderId="3" xfId="9">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="2" xfId="12" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="54">
@@ -2038,164 +2038,164 @@
         <v>1</v>
       </c>
       <c r="B2" s="28"/>
-      <c r="C2" s="97" t="s">
+      <c r="C2" s="93" t="s">
         <v>11</v>
       </c>
-      <c r="D2" s="98"/>
-      <c r="E2" s="101">
+      <c r="D2" s="94"/>
+      <c r="E2" s="97">
         <f>DATE(2025,8,12)</f>
         <v>45881</v>
       </c>
-      <c r="F2" s="101"/>
+      <c r="F2" s="97"/>
     </row>
     <row r="3" spans="1:121" s="26" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="24" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="99" t="s">
+      <c r="C3" s="95" t="s">
         <v>12</v>
       </c>
-      <c r="D3" s="100"/>
+      <c r="D3" s="96"/>
       <c r="E3" s="61">
         <v>1</v>
       </c>
       <c r="H3" s="62"/>
-      <c r="I3" s="88">
+      <c r="I3" s="99">
         <f>I4</f>
         <v>45880</v>
       </c>
-      <c r="J3" s="88"/>
-      <c r="K3" s="88"/>
-      <c r="L3" s="88"/>
-      <c r="M3" s="88"/>
-      <c r="N3" s="88">
+      <c r="J3" s="99"/>
+      <c r="K3" s="99"/>
+      <c r="L3" s="99"/>
+      <c r="M3" s="99"/>
+      <c r="N3" s="99">
         <f>N4</f>
         <v>45887</v>
       </c>
-      <c r="O3" s="88"/>
-      <c r="P3" s="88"/>
-      <c r="Q3" s="88"/>
-      <c r="R3" s="88"/>
-      <c r="S3" s="88">
+      <c r="O3" s="99"/>
+      <c r="P3" s="99"/>
+      <c r="Q3" s="99"/>
+      <c r="R3" s="99"/>
+      <c r="S3" s="99">
         <f>S4</f>
         <v>45894</v>
       </c>
-      <c r="T3" s="88"/>
-      <c r="U3" s="88"/>
-      <c r="V3" s="88"/>
-      <c r="W3" s="88"/>
-      <c r="X3" s="88">
+      <c r="T3" s="99"/>
+      <c r="U3" s="99"/>
+      <c r="V3" s="99"/>
+      <c r="W3" s="99"/>
+      <c r="X3" s="99">
         <f>X4</f>
         <v>45901</v>
       </c>
-      <c r="Y3" s="88"/>
-      <c r="Z3" s="88"/>
-      <c r="AA3" s="88"/>
-      <c r="AB3" s="88"/>
-      <c r="AC3" s="88">
+      <c r="Y3" s="99"/>
+      <c r="Z3" s="99"/>
+      <c r="AA3" s="99"/>
+      <c r="AB3" s="99"/>
+      <c r="AC3" s="99">
         <f t="shared" ref="AC3" si="0">AC4</f>
         <v>45908</v>
       </c>
-      <c r="AD3" s="88"/>
-      <c r="AE3" s="88"/>
-      <c r="AF3" s="88"/>
-      <c r="AG3" s="88"/>
-      <c r="AH3" s="88">
+      <c r="AD3" s="99"/>
+      <c r="AE3" s="99"/>
+      <c r="AF3" s="99"/>
+      <c r="AG3" s="99"/>
+      <c r="AH3" s="99">
         <f t="shared" ref="AH3" si="1">AH4</f>
         <v>45915</v>
       </c>
-      <c r="AI3" s="88"/>
-      <c r="AJ3" s="88"/>
-      <c r="AK3" s="88"/>
-      <c r="AL3" s="88"/>
-      <c r="AM3" s="88">
+      <c r="AI3" s="99"/>
+      <c r="AJ3" s="99"/>
+      <c r="AK3" s="99"/>
+      <c r="AL3" s="99"/>
+      <c r="AM3" s="99">
         <f t="shared" ref="AM3" si="2">AM4</f>
         <v>45922</v>
       </c>
-      <c r="AN3" s="88"/>
-      <c r="AO3" s="88"/>
-      <c r="AP3" s="88"/>
-      <c r="AQ3" s="88"/>
-      <c r="AR3" s="88">
+      <c r="AN3" s="99"/>
+      <c r="AO3" s="99"/>
+      <c r="AP3" s="99"/>
+      <c r="AQ3" s="99"/>
+      <c r="AR3" s="99">
         <f>AR4</f>
         <v>45929</v>
       </c>
-      <c r="AS3" s="88"/>
-      <c r="AT3" s="88"/>
-      <c r="AU3" s="88"/>
-      <c r="AV3" s="88"/>
-      <c r="AW3" s="88">
+      <c r="AS3" s="99"/>
+      <c r="AT3" s="99"/>
+      <c r="AU3" s="99"/>
+      <c r="AV3" s="99"/>
+      <c r="AW3" s="99">
         <f t="shared" ref="AW3" si="3">AW4</f>
         <v>45936</v>
       </c>
-      <c r="AX3" s="88"/>
-      <c r="AY3" s="88"/>
-      <c r="AZ3" s="88"/>
-      <c r="BA3" s="88"/>
-      <c r="BB3" s="88">
+      <c r="AX3" s="99"/>
+      <c r="AY3" s="99"/>
+      <c r="AZ3" s="99"/>
+      <c r="BA3" s="99"/>
+      <c r="BB3" s="99">
         <f t="shared" ref="BB3" si="4">BB4</f>
         <v>45943</v>
       </c>
-      <c r="BC3" s="88"/>
-      <c r="BD3" s="88"/>
-      <c r="BE3" s="88"/>
-      <c r="BF3" s="88"/>
-      <c r="BG3" s="88">
+      <c r="BC3" s="99"/>
+      <c r="BD3" s="99"/>
+      <c r="BE3" s="99"/>
+      <c r="BF3" s="99"/>
+      <c r="BG3" s="99">
         <f t="shared" ref="BG3" si="5">BG4</f>
         <v>45950</v>
       </c>
-      <c r="BH3" s="88"/>
-      <c r="BI3" s="88"/>
-      <c r="BJ3" s="88"/>
-      <c r="BK3" s="88"/>
-      <c r="BL3" s="88">
+      <c r="BH3" s="99"/>
+      <c r="BI3" s="99"/>
+      <c r="BJ3" s="99"/>
+      <c r="BK3" s="99"/>
+      <c r="BL3" s="99">
         <f t="shared" ref="BL3" si="6">BL4</f>
         <v>45957</v>
       </c>
-      <c r="BM3" s="88"/>
-      <c r="BN3" s="88"/>
-      <c r="BO3" s="88"/>
-      <c r="BP3" s="88"/>
-      <c r="BQ3" s="88">
+      <c r="BM3" s="99"/>
+      <c r="BN3" s="99"/>
+      <c r="BO3" s="99"/>
+      <c r="BP3" s="99"/>
+      <c r="BQ3" s="99">
         <f t="shared" ref="BQ3" si="7">BQ4</f>
         <v>45964</v>
       </c>
-      <c r="BR3" s="88"/>
-      <c r="BS3" s="88"/>
-      <c r="BT3" s="88"/>
-      <c r="BU3" s="88"/>
-      <c r="BV3" s="88">
+      <c r="BR3" s="99"/>
+      <c r="BS3" s="99"/>
+      <c r="BT3" s="99"/>
+      <c r="BU3" s="99"/>
+      <c r="BV3" s="99">
         <f t="shared" ref="BV3" si="8">BV4</f>
         <v>45971</v>
       </c>
-      <c r="BW3" s="88"/>
-      <c r="BX3" s="88"/>
-      <c r="BY3" s="88"/>
-      <c r="BZ3" s="88"/>
-      <c r="CA3" s="88">
+      <c r="BW3" s="99"/>
+      <c r="BX3" s="99"/>
+      <c r="BY3" s="99"/>
+      <c r="BZ3" s="99"/>
+      <c r="CA3" s="99">
         <f t="shared" ref="CA3" si="9">CA4</f>
         <v>45978</v>
       </c>
-      <c r="CB3" s="88"/>
-      <c r="CC3" s="88"/>
-      <c r="CD3" s="88"/>
-      <c r="CE3" s="88"/>
-      <c r="CF3" s="88">
+      <c r="CB3" s="99"/>
+      <c r="CC3" s="99"/>
+      <c r="CD3" s="99"/>
+      <c r="CE3" s="99"/>
+      <c r="CF3" s="99">
         <f t="shared" ref="CF3" si="10">CF4</f>
         <v>45985</v>
       </c>
-      <c r="CG3" s="88"/>
-      <c r="CH3" s="88"/>
-      <c r="CI3" s="88"/>
-      <c r="CJ3" s="88"/>
-      <c r="CK3" s="88">
+      <c r="CG3" s="99"/>
+      <c r="CH3" s="99"/>
+      <c r="CI3" s="99"/>
+      <c r="CJ3" s="99"/>
+      <c r="CK3" s="99">
         <f t="shared" ref="CK3" si="11">CK4</f>
         <v>45992</v>
       </c>
-      <c r="CL3" s="88"/>
-      <c r="CM3" s="88"/>
-      <c r="CN3" s="88"/>
-      <c r="CO3" s="89"/>
+      <c r="CL3" s="99"/>
+      <c r="CM3" s="99"/>
+      <c r="CN3" s="99"/>
+      <c r="CO3" s="100"/>
       <c r="CP3" s="84"/>
       <c r="CQ3" s="74"/>
       <c r="CR3" s="74"/>
@@ -3030,91 +3030,91 @@
         <f t="shared" ref="H7:H28" si="25">IF(OR(ISBLANK(task_start),ISBLANK(task_end)),"",task_end-task_start+1)</f>
         <v/>
       </c>
-      <c r="I7" s="90"/>
-      <c r="J7" s="91"/>
-      <c r="K7" s="91"/>
-      <c r="L7" s="91"/>
-      <c r="M7" s="91"/>
-      <c r="N7" s="91"/>
-      <c r="O7" s="91"/>
-      <c r="P7" s="91"/>
-      <c r="Q7" s="91"/>
-      <c r="R7" s="91"/>
-      <c r="S7" s="91"/>
-      <c r="T7" s="91"/>
-      <c r="U7" s="91"/>
-      <c r="V7" s="91"/>
-      <c r="W7" s="91"/>
-      <c r="X7" s="91"/>
-      <c r="Y7" s="91"/>
-      <c r="Z7" s="91"/>
-      <c r="AA7" s="91"/>
-      <c r="AB7" s="91"/>
-      <c r="AC7" s="91"/>
-      <c r="AD7" s="91"/>
-      <c r="AE7" s="91"/>
-      <c r="AF7" s="91"/>
-      <c r="AG7" s="91"/>
-      <c r="AH7" s="91"/>
-      <c r="AI7" s="91"/>
-      <c r="AJ7" s="91"/>
-      <c r="AK7" s="91"/>
-      <c r="AL7" s="91"/>
-      <c r="AM7" s="91"/>
-      <c r="AN7" s="91"/>
-      <c r="AO7" s="91"/>
-      <c r="AP7" s="91"/>
-      <c r="AQ7" s="91"/>
-      <c r="AR7" s="91"/>
-      <c r="AS7" s="91"/>
-      <c r="AT7" s="91"/>
-      <c r="AU7" s="91"/>
-      <c r="AV7" s="91"/>
-      <c r="AW7" s="91"/>
-      <c r="AX7" s="91"/>
-      <c r="AY7" s="91"/>
-      <c r="AZ7" s="91"/>
-      <c r="BA7" s="91"/>
-      <c r="BB7" s="91"/>
-      <c r="BC7" s="91"/>
-      <c r="BD7" s="91"/>
-      <c r="BE7" s="91"/>
-      <c r="BF7" s="91"/>
-      <c r="BG7" s="91"/>
-      <c r="BH7" s="91"/>
-      <c r="BI7" s="91"/>
-      <c r="BJ7" s="91"/>
-      <c r="BK7" s="91"/>
-      <c r="BL7" s="91"/>
-      <c r="BM7" s="91"/>
-      <c r="BN7" s="91"/>
-      <c r="BO7" s="91"/>
-      <c r="BP7" s="91"/>
-      <c r="BQ7" s="91"/>
-      <c r="BR7" s="91"/>
-      <c r="BS7" s="91"/>
-      <c r="BT7" s="91"/>
-      <c r="BU7" s="91"/>
-      <c r="BV7" s="91"/>
-      <c r="BW7" s="91"/>
-      <c r="BX7" s="91"/>
-      <c r="BY7" s="91"/>
-      <c r="BZ7" s="91"/>
-      <c r="CA7" s="91"/>
-      <c r="CB7" s="91"/>
-      <c r="CC7" s="91"/>
-      <c r="CD7" s="91"/>
-      <c r="CE7" s="91"/>
-      <c r="CF7" s="91"/>
-      <c r="CG7" s="91"/>
-      <c r="CH7" s="91"/>
-      <c r="CI7" s="91"/>
-      <c r="CJ7" s="91"/>
-      <c r="CK7" s="91"/>
-      <c r="CL7" s="91"/>
-      <c r="CM7" s="91"/>
-      <c r="CN7" s="91"/>
-      <c r="CO7" s="91"/>
+      <c r="I7" s="101"/>
+      <c r="J7" s="102"/>
+      <c r="K7" s="102"/>
+      <c r="L7" s="102"/>
+      <c r="M7" s="102"/>
+      <c r="N7" s="102"/>
+      <c r="O7" s="102"/>
+      <c r="P7" s="102"/>
+      <c r="Q7" s="102"/>
+      <c r="R7" s="102"/>
+      <c r="S7" s="102"/>
+      <c r="T7" s="102"/>
+      <c r="U7" s="102"/>
+      <c r="V7" s="102"/>
+      <c r="W7" s="102"/>
+      <c r="X7" s="102"/>
+      <c r="Y7" s="102"/>
+      <c r="Z7" s="102"/>
+      <c r="AA7" s="102"/>
+      <c r="AB7" s="102"/>
+      <c r="AC7" s="102"/>
+      <c r="AD7" s="102"/>
+      <c r="AE7" s="102"/>
+      <c r="AF7" s="102"/>
+      <c r="AG7" s="102"/>
+      <c r="AH7" s="102"/>
+      <c r="AI7" s="102"/>
+      <c r="AJ7" s="102"/>
+      <c r="AK7" s="102"/>
+      <c r="AL7" s="102"/>
+      <c r="AM7" s="102"/>
+      <c r="AN7" s="102"/>
+      <c r="AO7" s="102"/>
+      <c r="AP7" s="102"/>
+      <c r="AQ7" s="102"/>
+      <c r="AR7" s="102"/>
+      <c r="AS7" s="102"/>
+      <c r="AT7" s="102"/>
+      <c r="AU7" s="102"/>
+      <c r="AV7" s="102"/>
+      <c r="AW7" s="102"/>
+      <c r="AX7" s="102"/>
+      <c r="AY7" s="102"/>
+      <c r="AZ7" s="102"/>
+      <c r="BA7" s="102"/>
+      <c r="BB7" s="102"/>
+      <c r="BC7" s="102"/>
+      <c r="BD7" s="102"/>
+      <c r="BE7" s="102"/>
+      <c r="BF7" s="102"/>
+      <c r="BG7" s="102"/>
+      <c r="BH7" s="102"/>
+      <c r="BI7" s="102"/>
+      <c r="BJ7" s="102"/>
+      <c r="BK7" s="102"/>
+      <c r="BL7" s="102"/>
+      <c r="BM7" s="102"/>
+      <c r="BN7" s="102"/>
+      <c r="BO7" s="102"/>
+      <c r="BP7" s="102"/>
+      <c r="BQ7" s="102"/>
+      <c r="BR7" s="102"/>
+      <c r="BS7" s="102"/>
+      <c r="BT7" s="102"/>
+      <c r="BU7" s="102"/>
+      <c r="BV7" s="102"/>
+      <c r="BW7" s="102"/>
+      <c r="BX7" s="102"/>
+      <c r="BY7" s="102"/>
+      <c r="BZ7" s="102"/>
+      <c r="CA7" s="102"/>
+      <c r="CB7" s="102"/>
+      <c r="CC7" s="102"/>
+      <c r="CD7" s="102"/>
+      <c r="CE7" s="102"/>
+      <c r="CF7" s="102"/>
+      <c r="CG7" s="102"/>
+      <c r="CH7" s="102"/>
+      <c r="CI7" s="102"/>
+      <c r="CJ7" s="102"/>
+      <c r="CK7" s="102"/>
+      <c r="CL7" s="102"/>
+      <c r="CM7" s="102"/>
+      <c r="CN7" s="102"/>
+      <c r="CO7" s="102"/>
       <c r="CP7" s="87"/>
       <c r="CQ7" s="78"/>
       <c r="CR7" s="78"/>
@@ -3148,10 +3148,10 @@
       <c r="A8" s="24" t="s">
         <v>6</v>
       </c>
-      <c r="B8" s="102" t="s">
+      <c r="B8" s="98" t="s">
         <v>29</v>
       </c>
-      <c r="C8" s="102"/>
+      <c r="C8" s="98"/>
       <c r="D8" s="13">
         <v>1</v>
       </c>
@@ -3282,10 +3282,10 @@
     </row>
     <row r="9" spans="1:121" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="24"/>
-      <c r="B9" s="102" t="s">
+      <c r="B9" s="98" t="s">
         <v>30</v>
       </c>
-      <c r="C9" s="102"/>
+      <c r="C9" s="98"/>
       <c r="D9" s="13">
         <v>1</v>
       </c>
@@ -3413,10 +3413,10 @@
     </row>
     <row r="10" spans="1:121" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="23"/>
-      <c r="B10" s="102" t="s">
+      <c r="B10" s="98" t="s">
         <v>31</v>
       </c>
-      <c r="C10" s="102"/>
+      <c r="C10" s="98"/>
       <c r="D10" s="13">
         <v>1</v>
       </c>
@@ -3547,10 +3547,10 @@
     </row>
     <row r="11" spans="1:121" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="23"/>
-      <c r="B11" s="102" t="s">
+      <c r="B11" s="98" t="s">
         <v>38</v>
       </c>
-      <c r="C11" s="102"/>
+      <c r="C11" s="98"/>
       <c r="D11" s="13">
         <v>1</v>
       </c>
@@ -3678,10 +3678,10 @@
     </row>
     <row r="12" spans="1:121" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="23"/>
-      <c r="B12" s="102" t="s">
+      <c r="B12" s="98" t="s">
         <v>39</v>
       </c>
-      <c r="C12" s="102"/>
+      <c r="C12" s="98"/>
       <c r="D12" s="13">
         <v>1</v>
       </c>
@@ -3810,10 +3810,10 @@
     </row>
     <row r="13" spans="1:121" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="23"/>
-      <c r="B13" s="102" t="s">
+      <c r="B13" s="98" t="s">
         <v>40</v>
       </c>
-      <c r="C13" s="102"/>
+      <c r="C13" s="98"/>
       <c r="D13" s="13">
         <v>1</v>
       </c>
@@ -3955,91 +3955,91 @@
         <f t="shared" si="25"/>
         <v/>
       </c>
-      <c r="I14" s="94"/>
-      <c r="J14" s="95"/>
-      <c r="K14" s="95"/>
-      <c r="L14" s="95"/>
-      <c r="M14" s="95"/>
-      <c r="N14" s="95"/>
-      <c r="O14" s="95"/>
-      <c r="P14" s="95"/>
-      <c r="Q14" s="95"/>
-      <c r="R14" s="95"/>
-      <c r="S14" s="95"/>
-      <c r="T14" s="95"/>
-      <c r="U14" s="95"/>
-      <c r="V14" s="95"/>
-      <c r="W14" s="95"/>
-      <c r="X14" s="95"/>
-      <c r="Y14" s="95"/>
-      <c r="Z14" s="95"/>
-      <c r="AA14" s="95"/>
-      <c r="AB14" s="95"/>
-      <c r="AC14" s="95"/>
-      <c r="AD14" s="95"/>
-      <c r="AE14" s="95"/>
-      <c r="AF14" s="95"/>
-      <c r="AG14" s="95"/>
-      <c r="AH14" s="95"/>
-      <c r="AI14" s="95"/>
-      <c r="AJ14" s="95"/>
-      <c r="AK14" s="95"/>
-      <c r="AL14" s="95"/>
-      <c r="AM14" s="95"/>
-      <c r="AN14" s="95"/>
-      <c r="AO14" s="95"/>
-      <c r="AP14" s="95"/>
-      <c r="AQ14" s="95"/>
-      <c r="AR14" s="95"/>
-      <c r="AS14" s="95"/>
-      <c r="AT14" s="95"/>
-      <c r="AU14" s="95"/>
-      <c r="AV14" s="95"/>
-      <c r="AW14" s="95"/>
-      <c r="AX14" s="95"/>
-      <c r="AY14" s="95"/>
-      <c r="AZ14" s="95"/>
-      <c r="BA14" s="95"/>
-      <c r="BB14" s="95"/>
-      <c r="BC14" s="95"/>
-      <c r="BD14" s="95"/>
-      <c r="BE14" s="95"/>
-      <c r="BF14" s="95"/>
-      <c r="BG14" s="95"/>
-      <c r="BH14" s="95"/>
-      <c r="BI14" s="95"/>
-      <c r="BJ14" s="95"/>
-      <c r="BK14" s="95"/>
-      <c r="BL14" s="95"/>
-      <c r="BM14" s="95"/>
-      <c r="BN14" s="95"/>
-      <c r="BO14" s="95"/>
-      <c r="BP14" s="95"/>
-      <c r="BQ14" s="95"/>
-      <c r="BR14" s="95"/>
-      <c r="BS14" s="95"/>
-      <c r="BT14" s="95"/>
-      <c r="BU14" s="95"/>
-      <c r="BV14" s="95"/>
-      <c r="BW14" s="95"/>
-      <c r="BX14" s="95"/>
-      <c r="BY14" s="95"/>
-      <c r="BZ14" s="95"/>
-      <c r="CA14" s="95"/>
-      <c r="CB14" s="95"/>
-      <c r="CC14" s="95"/>
-      <c r="CD14" s="95"/>
-      <c r="CE14" s="95"/>
-      <c r="CF14" s="95"/>
-      <c r="CG14" s="95"/>
-      <c r="CH14" s="95"/>
-      <c r="CI14" s="95"/>
-      <c r="CJ14" s="95"/>
-      <c r="CK14" s="95"/>
-      <c r="CL14" s="95"/>
-      <c r="CM14" s="95"/>
-      <c r="CN14" s="95"/>
-      <c r="CO14" s="96"/>
+      <c r="I14" s="90"/>
+      <c r="J14" s="91"/>
+      <c r="K14" s="91"/>
+      <c r="L14" s="91"/>
+      <c r="M14" s="91"/>
+      <c r="N14" s="91"/>
+      <c r="O14" s="91"/>
+      <c r="P14" s="91"/>
+      <c r="Q14" s="91"/>
+      <c r="R14" s="91"/>
+      <c r="S14" s="91"/>
+      <c r="T14" s="91"/>
+      <c r="U14" s="91"/>
+      <c r="V14" s="91"/>
+      <c r="W14" s="91"/>
+      <c r="X14" s="91"/>
+      <c r="Y14" s="91"/>
+      <c r="Z14" s="91"/>
+      <c r="AA14" s="91"/>
+      <c r="AB14" s="91"/>
+      <c r="AC14" s="91"/>
+      <c r="AD14" s="91"/>
+      <c r="AE14" s="91"/>
+      <c r="AF14" s="91"/>
+      <c r="AG14" s="91"/>
+      <c r="AH14" s="91"/>
+      <c r="AI14" s="91"/>
+      <c r="AJ14" s="91"/>
+      <c r="AK14" s="91"/>
+      <c r="AL14" s="91"/>
+      <c r="AM14" s="91"/>
+      <c r="AN14" s="91"/>
+      <c r="AO14" s="91"/>
+      <c r="AP14" s="91"/>
+      <c r="AQ14" s="91"/>
+      <c r="AR14" s="91"/>
+      <c r="AS14" s="91"/>
+      <c r="AT14" s="91"/>
+      <c r="AU14" s="91"/>
+      <c r="AV14" s="91"/>
+      <c r="AW14" s="91"/>
+      <c r="AX14" s="91"/>
+      <c r="AY14" s="91"/>
+      <c r="AZ14" s="91"/>
+      <c r="BA14" s="91"/>
+      <c r="BB14" s="91"/>
+      <c r="BC14" s="91"/>
+      <c r="BD14" s="91"/>
+      <c r="BE14" s="91"/>
+      <c r="BF14" s="91"/>
+      <c r="BG14" s="91"/>
+      <c r="BH14" s="91"/>
+      <c r="BI14" s="91"/>
+      <c r="BJ14" s="91"/>
+      <c r="BK14" s="91"/>
+      <c r="BL14" s="91"/>
+      <c r="BM14" s="91"/>
+      <c r="BN14" s="91"/>
+      <c r="BO14" s="91"/>
+      <c r="BP14" s="91"/>
+      <c r="BQ14" s="91"/>
+      <c r="BR14" s="91"/>
+      <c r="BS14" s="91"/>
+      <c r="BT14" s="91"/>
+      <c r="BU14" s="91"/>
+      <c r="BV14" s="91"/>
+      <c r="BW14" s="91"/>
+      <c r="BX14" s="91"/>
+      <c r="BY14" s="91"/>
+      <c r="BZ14" s="91"/>
+      <c r="CA14" s="91"/>
+      <c r="CB14" s="91"/>
+      <c r="CC14" s="91"/>
+      <c r="CD14" s="91"/>
+      <c r="CE14" s="91"/>
+      <c r="CF14" s="91"/>
+      <c r="CG14" s="91"/>
+      <c r="CH14" s="91"/>
+      <c r="CI14" s="91"/>
+      <c r="CJ14" s="91"/>
+      <c r="CK14" s="91"/>
+      <c r="CL14" s="91"/>
+      <c r="CM14" s="91"/>
+      <c r="CN14" s="91"/>
+      <c r="CO14" s="92"/>
       <c r="CP14" s="86"/>
       <c r="CQ14"/>
       <c r="CR14"/>
@@ -4207,7 +4207,7 @@
       </c>
       <c r="C16" s="30"/>
       <c r="D16" s="16">
-        <v>0.3</v>
+        <v>0.55000000000000004</v>
       </c>
       <c r="E16" s="42">
         <v>45922</v>
@@ -4338,7 +4338,7 @@
       </c>
       <c r="C17" s="30"/>
       <c r="D17" s="16">
-        <v>0.6</v>
+        <v>0.85</v>
       </c>
       <c r="E17" s="42">
         <v>45926</v>
@@ -5002,91 +5002,91 @@
         <f t="shared" si="25"/>
         <v/>
       </c>
-      <c r="I22" s="92"/>
-      <c r="J22" s="93"/>
-      <c r="K22" s="93"/>
-      <c r="L22" s="93"/>
-      <c r="M22" s="93"/>
-      <c r="N22" s="93"/>
-      <c r="O22" s="93"/>
-      <c r="P22" s="93"/>
-      <c r="Q22" s="93"/>
-      <c r="R22" s="93"/>
-      <c r="S22" s="93"/>
-      <c r="T22" s="93"/>
-      <c r="U22" s="93"/>
-      <c r="V22" s="93"/>
-      <c r="W22" s="93"/>
-      <c r="X22" s="93"/>
-      <c r="Y22" s="93"/>
-      <c r="Z22" s="93"/>
-      <c r="AA22" s="93"/>
-      <c r="AB22" s="93"/>
-      <c r="AC22" s="93"/>
-      <c r="AD22" s="93"/>
-      <c r="AE22" s="93"/>
-      <c r="AF22" s="93"/>
-      <c r="AG22" s="93"/>
-      <c r="AH22" s="93"/>
-      <c r="AI22" s="93"/>
-      <c r="AJ22" s="93"/>
-      <c r="AK22" s="93"/>
-      <c r="AL22" s="93"/>
-      <c r="AM22" s="93"/>
-      <c r="AN22" s="93"/>
-      <c r="AO22" s="93"/>
-      <c r="AP22" s="93"/>
-      <c r="AQ22" s="93"/>
-      <c r="AR22" s="93"/>
-      <c r="AS22" s="93"/>
-      <c r="AT22" s="93"/>
-      <c r="AU22" s="93"/>
-      <c r="AV22" s="93"/>
-      <c r="AW22" s="93"/>
-      <c r="AX22" s="93"/>
-      <c r="AY22" s="93"/>
-      <c r="AZ22" s="93"/>
-      <c r="BA22" s="93"/>
-      <c r="BB22" s="93"/>
-      <c r="BC22" s="93"/>
-      <c r="BD22" s="93"/>
-      <c r="BE22" s="93"/>
-      <c r="BF22" s="93"/>
-      <c r="BG22" s="93"/>
-      <c r="BH22" s="93"/>
-      <c r="BI22" s="93"/>
-      <c r="BJ22" s="93"/>
-      <c r="BK22" s="93"/>
-      <c r="BL22" s="93"/>
-      <c r="BM22" s="93"/>
-      <c r="BN22" s="93"/>
-      <c r="BO22" s="93"/>
-      <c r="BP22" s="93"/>
-      <c r="BQ22" s="93"/>
-      <c r="BR22" s="93"/>
-      <c r="BS22" s="93"/>
-      <c r="BT22" s="93"/>
-      <c r="BU22" s="93"/>
-      <c r="BV22" s="93"/>
-      <c r="BW22" s="93"/>
-      <c r="BX22" s="93"/>
-      <c r="BY22" s="93"/>
-      <c r="BZ22" s="93"/>
-      <c r="CA22" s="93"/>
-      <c r="CB22" s="93"/>
-      <c r="CC22" s="93"/>
-      <c r="CD22" s="93"/>
-      <c r="CE22" s="93"/>
-      <c r="CF22" s="93"/>
-      <c r="CG22" s="93"/>
-      <c r="CH22" s="93"/>
-      <c r="CI22" s="93"/>
-      <c r="CJ22" s="93"/>
-      <c r="CK22" s="93"/>
-      <c r="CL22" s="93"/>
-      <c r="CM22" s="93"/>
-      <c r="CN22" s="93"/>
-      <c r="CO22" s="93"/>
+      <c r="I22" s="88"/>
+      <c r="J22" s="89"/>
+      <c r="K22" s="89"/>
+      <c r="L22" s="89"/>
+      <c r="M22" s="89"/>
+      <c r="N22" s="89"/>
+      <c r="O22" s="89"/>
+      <c r="P22" s="89"/>
+      <c r="Q22" s="89"/>
+      <c r="R22" s="89"/>
+      <c r="S22" s="89"/>
+      <c r="T22" s="89"/>
+      <c r="U22" s="89"/>
+      <c r="V22" s="89"/>
+      <c r="W22" s="89"/>
+      <c r="X22" s="89"/>
+      <c r="Y22" s="89"/>
+      <c r="Z22" s="89"/>
+      <c r="AA22" s="89"/>
+      <c r="AB22" s="89"/>
+      <c r="AC22" s="89"/>
+      <c r="AD22" s="89"/>
+      <c r="AE22" s="89"/>
+      <c r="AF22" s="89"/>
+      <c r="AG22" s="89"/>
+      <c r="AH22" s="89"/>
+      <c r="AI22" s="89"/>
+      <c r="AJ22" s="89"/>
+      <c r="AK22" s="89"/>
+      <c r="AL22" s="89"/>
+      <c r="AM22" s="89"/>
+      <c r="AN22" s="89"/>
+      <c r="AO22" s="89"/>
+      <c r="AP22" s="89"/>
+      <c r="AQ22" s="89"/>
+      <c r="AR22" s="89"/>
+      <c r="AS22" s="89"/>
+      <c r="AT22" s="89"/>
+      <c r="AU22" s="89"/>
+      <c r="AV22" s="89"/>
+      <c r="AW22" s="89"/>
+      <c r="AX22" s="89"/>
+      <c r="AY22" s="89"/>
+      <c r="AZ22" s="89"/>
+      <c r="BA22" s="89"/>
+      <c r="BB22" s="89"/>
+      <c r="BC22" s="89"/>
+      <c r="BD22" s="89"/>
+      <c r="BE22" s="89"/>
+      <c r="BF22" s="89"/>
+      <c r="BG22" s="89"/>
+      <c r="BH22" s="89"/>
+      <c r="BI22" s="89"/>
+      <c r="BJ22" s="89"/>
+      <c r="BK22" s="89"/>
+      <c r="BL22" s="89"/>
+      <c r="BM22" s="89"/>
+      <c r="BN22" s="89"/>
+      <c r="BO22" s="89"/>
+      <c r="BP22" s="89"/>
+      <c r="BQ22" s="89"/>
+      <c r="BR22" s="89"/>
+      <c r="BS22" s="89"/>
+      <c r="BT22" s="89"/>
+      <c r="BU22" s="89"/>
+      <c r="BV22" s="89"/>
+      <c r="BW22" s="89"/>
+      <c r="BX22" s="89"/>
+      <c r="BY22" s="89"/>
+      <c r="BZ22" s="89"/>
+      <c r="CA22" s="89"/>
+      <c r="CB22" s="89"/>
+      <c r="CC22" s="89"/>
+      <c r="CD22" s="89"/>
+      <c r="CE22" s="89"/>
+      <c r="CF22" s="89"/>
+      <c r="CG22" s="89"/>
+      <c r="CH22" s="89"/>
+      <c r="CI22" s="89"/>
+      <c r="CJ22" s="89"/>
+      <c r="CK22" s="89"/>
+      <c r="CL22" s="89"/>
+      <c r="CM22" s="89"/>
+      <c r="CN22" s="89"/>
+      <c r="CO22" s="89"/>
       <c r="CP22" s="86"/>
       <c r="CQ22"/>
       <c r="CR22"/>
@@ -6788,6 +6788,19 @@
     </row>
   </sheetData>
   <mergeCells count="29">
+    <mergeCell ref="CF3:CJ3"/>
+    <mergeCell ref="CK3:CO3"/>
+    <mergeCell ref="I7:CO7"/>
+    <mergeCell ref="BB3:BF3"/>
+    <mergeCell ref="BG3:BK3"/>
+    <mergeCell ref="BL3:BP3"/>
+    <mergeCell ref="BQ3:BU3"/>
+    <mergeCell ref="BV3:BZ3"/>
+    <mergeCell ref="AC3:AG3"/>
+    <mergeCell ref="AH3:AL3"/>
+    <mergeCell ref="AM3:AQ3"/>
+    <mergeCell ref="AR3:AV3"/>
+    <mergeCell ref="AW3:BA3"/>
     <mergeCell ref="I22:CO22"/>
     <mergeCell ref="I14:CO14"/>
     <mergeCell ref="C2:D2"/>
@@ -6804,19 +6817,6 @@
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B12:C12"/>
     <mergeCell ref="CA3:CE3"/>
-    <mergeCell ref="CF3:CJ3"/>
-    <mergeCell ref="CK3:CO3"/>
-    <mergeCell ref="I7:CO7"/>
-    <mergeCell ref="BB3:BF3"/>
-    <mergeCell ref="BG3:BK3"/>
-    <mergeCell ref="BL3:BP3"/>
-    <mergeCell ref="BQ3:BU3"/>
-    <mergeCell ref="BV3:BZ3"/>
-    <mergeCell ref="AC3:AG3"/>
-    <mergeCell ref="AH3:AL3"/>
-    <mergeCell ref="AM3:AQ3"/>
-    <mergeCell ref="AR3:AV3"/>
-    <mergeCell ref="AW3:BA3"/>
   </mergeCells>
   <conditionalFormatting sqref="D6:D35">
     <cfRule type="dataBar" priority="17">
@@ -7191,6 +7191,15 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
@@ -7208,15 +7217,6 @@
     <MediaServiceKeyPoints xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -7241,6 +7241,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E4A34E49-7289-4AEA-9593-4F55E04ADB10}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AC3AD2E1-977A-4D4F-8EE8-D64B5FFADF75}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -7250,12 +7258,4 @@
     <ds:schemaRef ds:uri="230e9df3-be65-4c73-a93b-d1236ebd677e"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E4A34E49-7289-4AEA-9593-4F55E04ADB10}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>